<commit_message>
Update berita 2026-08-05 05:13 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-07-30.xlsx
+++ b/data/berita_2026-07-30.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -512,8 +512,84 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>6 titik shuttle bus gratis GIIAS 2026 ke ICE BSD, cek lokasi &amp; jadwalnya</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Thu, 30 Jul 2026 18:17:21 +0700</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Penyelenggara GAIKINDO Indonesia International Auto Show (GIIAS) 2026 kembali menyediakan layanan shuttle bus gratis ...</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5672876/6-titik-shuttle-bus-gratis-giias-2026-ke-ice-bsd-cek-lokasi-jadwalnya</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/IMG_1404.jpg</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Hiburan</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Sinopsis Spider-Man: Brand New Day, film baru Tom Holland yang resmi tayang di bioskop</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Thu, 30 Jul 2026 23:22:19 +0700</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Kabar gembira bagi para penggemar film superhero. Spider-Man: Brand New Day resmi tayang di bioskop mulai 30 Juli 2026, ...</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5673487/sinopsis-spider-man-brand-new-day-film-baru-tom-holland-yang-resmi-tayang-di-bioskop</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/18/7297.jpg</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H2"/>
+  <autoFilter ref="A1:H4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>